<commit_message>
auto: snapshot 2026-09-13 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -67,6 +67,7 @@
     <sheet name="2026-09-10" sheetId="58" state="visible" r:id="rId58"/>
     <sheet name="2026-09-11" sheetId="59" state="visible" r:id="rId59"/>
     <sheet name="2026-09-12" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="2026-09-13" sheetId="61" state="visible" r:id="rId61"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47925,6 +47926,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-13 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>12044</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+8367</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8383</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4510</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1461</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>10804</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>11439</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>10872</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>9673</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10828</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>10913</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>10842</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>10715</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8976</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7648</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+3746</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7152</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3902</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>10568</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3677</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>4682</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10771</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10624</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10759</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10429</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10444</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>8322</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4560</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-14 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -68,6 +68,7 @@
     <sheet name="2026-09-11" sheetId="59" state="visible" r:id="rId59"/>
     <sheet name="2026-09-12" sheetId="60" state="visible" r:id="rId60"/>
     <sheet name="2026-09-13" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="2026-09-14" sheetId="62" state="visible" r:id="rId62"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48805,6 +48806,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-14 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>12044</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+8367</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8383</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4510</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1461</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>10804</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>11439</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>10872</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>9673</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10828</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>10913</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>10842</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>10715</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8976</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7648</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+3746</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7152</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3902</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>10568</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3677</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>4682</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10771</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10624</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10759</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10429</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10444</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>8322</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4560</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-15 13:01:02
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -69,6 +69,7 @@
     <sheet name="2026-09-12" sheetId="60" state="visible" r:id="rId60"/>
     <sheet name="2026-09-13" sheetId="61" state="visible" r:id="rId61"/>
     <sheet name="2026-09-14" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="2026-09-15" sheetId="63" state="visible" r:id="rId63"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -49685,6 +49686,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-15 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>12044</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+8367</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8383</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4510</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1461</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>10804</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>11439</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>10872</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>9673</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10828</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>10913</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>10842</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>10715</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8976</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7648</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+3746</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7152</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3902</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>10568</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3677</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>4682</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10771</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10624</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10759</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10429</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10444</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>8322</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4560</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-16 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -70,6 +70,7 @@
     <sheet name="2026-09-13" sheetId="61" state="visible" r:id="rId61"/>
     <sheet name="2026-09-14" sheetId="62" state="visible" r:id="rId62"/>
     <sheet name="2026-09-15" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="2026-09-16" sheetId="64" state="visible" r:id="rId64"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -50565,6 +50566,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-16 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>12044</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+8367</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8383</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4510</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1461</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>10804</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>11439</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>10872</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>9673</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10828</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>10913</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>10842</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>10715</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8976</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7648</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+3746</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7152</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3902</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>10568</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3677</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>4682</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10771</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10624</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10759</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10429</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10444</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>8322</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4560</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-17 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -71,6 +71,7 @@
     <sheet name="2026-09-14" sheetId="62" state="visible" r:id="rId62"/>
     <sheet name="2026-09-15" sheetId="63" state="visible" r:id="rId63"/>
     <sheet name="2026-09-16" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="2026-09-17" sheetId="65" state="visible" r:id="rId65"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -51445,6 +51446,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-17 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>12044</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+8367</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8383</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4510</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1461</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>10804</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>11439</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>10872</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>9673</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10828</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>10913</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>10842</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>10715</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8976</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7648</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+3746</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7152</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3902</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>10568</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3677</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>4682</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10771</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10624</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10759</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10429</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10444</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>8322</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4560</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-18 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -72,6 +72,7 @@
     <sheet name="2026-09-15" sheetId="63" state="visible" r:id="rId63"/>
     <sheet name="2026-09-16" sheetId="64" state="visible" r:id="rId64"/>
     <sheet name="2026-09-17" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="2026-09-18" sheetId="66" state="visible" r:id="rId66"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -52325,6 +52326,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-18 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>12044</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+8367</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8383</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4510</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1461</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>10804</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>11439</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>10872</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>9673</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10828</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>10913</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>10842</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>10715</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8976</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7648</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+3746</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7152</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3902</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>10568</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3677</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>4682</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>10771</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10624</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10759</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10429</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10444</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>8322</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>4560</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-19 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -73,6 +73,7 @@
     <sheet name="2026-09-16" sheetId="64" state="visible" r:id="rId64"/>
     <sheet name="2026-09-17" sheetId="65" state="visible" r:id="rId65"/>
     <sheet name="2026-09-18" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="2026-09-19" sheetId="67" state="visible" r:id="rId67"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -53190,6 +53191,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-19 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>12044</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+8367</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8383</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4510</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1461</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>10804</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>11439</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>10872</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>9673</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10828</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>10913</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>10842</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>10715</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8976</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7648</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+3746</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7152</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3902</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>10568</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3677</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>4682</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>10771</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10624</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10759</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10429</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10444</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>8322</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>4560</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-20 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -74,6 +74,7 @@
     <sheet name="2026-09-17" sheetId="65" state="visible" r:id="rId65"/>
     <sheet name="2026-09-18" sheetId="66" state="visible" r:id="rId66"/>
     <sheet name="2026-09-19" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="2026-09-20" sheetId="68" state="visible" r:id="rId68"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -54055,6 +54056,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-20 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>17694</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+14017</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>14213</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+5830</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>10160</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+7111</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>16200</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+5396</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>17269</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+5830</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>16702</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+5830</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>15454</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+5781</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>16298</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+5470</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>16563</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+5650</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>16492</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+5650</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>16386</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+5671</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>14806</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+5830</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>13228</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+9326</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>12622</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+5470</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>9552</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+5650</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>16141</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+5573</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>9180</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+5503</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>5432</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>16344</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+5573</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>16344</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+5720</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>16479</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+5720</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>16114</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+5685</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>16164</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+5720</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>13673</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+5351</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>5310</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>